<commit_message>
preparacion para regulacion ocultar fantasma despacho
</commit_message>
<xml_diff>
--- a/saldos_iniciales.xlsx
+++ b/saldos_iniciales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d57f09bfa23d157f/Desktop/PROYECTO_ALMACEN/Pasantias2026-Proyecto-Almacen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{525F1C35-017A-478D-B5D7-B8BBD40CBFB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{525F1C35-017A-478D-B5D7-B8BBD40CBFB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1FCBCA3-BDA0-43FA-976E-5BE18F665F59}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{EA8C7E67-04D3-4A49-B8B2-FB7ADE20D45A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>CANTIDAD</t>
   </si>
@@ -66,22 +66,16 @@
     <t>N/P</t>
   </si>
   <si>
-    <t>01404090083</t>
-  </si>
-  <si>
     <t>STOCK LOTE</t>
   </si>
   <si>
-    <t>prueba</t>
+    <t>CÓDIGO</t>
   </si>
   <si>
-    <t>mantenimiento</t>
+    <t>TIPO</t>
   </si>
   <si>
-    <t>US$</t>
-  </si>
-  <si>
-    <t>CÓDIGO</t>
+    <t>U.M</t>
   </si>
 </sst>
 </file>
@@ -89,7 +83,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -140,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -148,8 +142,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +463,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="40.28515625" customWidth="1"/>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
     <col min="4" max="4" width="24.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
@@ -484,102 +477,63 @@
     <col min="14" max="14" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>12</v>
+      <c r="C1" t="s">
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>14</v>
+      <c r="M1" s="1" t="s">
+        <v>13</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>123</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2">
-        <v>5</v>
-      </c>
-      <c r="J2">
-        <v>5</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>10</v>
-      </c>
-      <c r="M2" s="4">
-        <v>42851</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="O2" s="3"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>

</xml_diff>